<commit_message>
Ganti nama kode strategi: PB → TP, BO → TB, MR → PJ (tanpa perubahan perilaku)
Penggantian mekanis di kode, uji, config, SPEC, README, dan contoh: kode strategi, kode aturan
(PB1 → TP1, dst.), bagian config strategi.pb/bo/mr → strategi.tp/tb/pj, nama run backtest, dan
berkas uji strategi. Berkas acuan E2E dibangkitkan ulang (hanya nama kode dan hash8 berubah).
Perilaku belum berubah; aturan tren turun menyusul pada commit berikutnya. Semua uji lulus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HXtTE2q4GGWxFy6EkHmbcn
</commit_message>
<xml_diff>
--- a/tests/fixtures/e2e/acuan/rencana.xlsx
+++ b/tests/fixtures/e2e/acuan/rencana.xlsx
@@ -453,7 +453,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dibuat: 2025-09-10 20:00:00 WIB — hash8 44b5deb5 — versi 0.1.0 — REPLAY (--tanggal)</t>
+          <t>Dibuat: 2025-09-10 20:00:00 WIB — hash8 2d1ece58 — versi 0.1.0 — REPLAY (--tanggal)</t>
         </is>
       </c>
     </row>
@@ -745,7 +745,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -826,7 +826,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1038,7 +1038,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>TP</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2244,21 +2244,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Penyimpangan PB: sampel jurnal 0 &lt; 20: belum diuji</t>
+          <t>Penyimpangan TP: sampel jurnal 0 &lt; 20: belum diuji</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Penyimpangan BO: sampel jurnal 0 &lt; 20: belum diuji</t>
+          <t>Penyimpangan TB: sampel jurnal 0 &lt; 20: belum diuji</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Penyimpangan MR: sampel jurnal 0 &lt; 20: belum diuji</t>
+          <t>Penyimpangan PJ: sampel jurnal 0 &lt; 20: belum diuji</t>
         </is>
       </c>
     </row>

</xml_diff>